<commit_message>
added all source code from griffiths text book.
</commit_message>
<xml_diff>
--- a/inputs/slope/input_template_griffiths1_6.xlsx
+++ b/inputs/slope/input_template_griffiths1_6.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/cursor_projects/xslope/inputs/slope/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D0936D3-AC1D-7745-ADF3-3CA4685F085C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3645DF27-2956-2642-AD26-83DB99DC405B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32240" yWindow="3440" windowWidth="36380" windowHeight="18420" activeTab="3" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="33040" yWindow="1360" windowWidth="34660" windowHeight="19780" activeTab="3" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -859,7 +859,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -992,6 +992,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -6413,11 +6416,11 @@
       <c r="T4" s="3"/>
       <c r="U4" s="3"/>
       <c r="V4" s="3"/>
-      <c r="W4" s="1">
+      <c r="W4" s="50">
         <v>700000</v>
       </c>
       <c r="X4" s="3">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
refactored the code in fem.py to restore sign convesion where tension = positive and compression = negative. This makes it consistent with griffiths and lane 1999 paper and the standard FEM stress strain equations.
</commit_message>
<xml_diff>
--- a/inputs/slope/input_template_griffiths1_6.xlsx
+++ b/inputs/slope/input_template_griffiths1_6.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/cursor_projects/xslope/inputs/slope/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3645DF27-2956-2642-AD26-83DB99DC405B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D73E5FF-D079-8D47-A1DE-9C0E17D23B11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33040" yWindow="1360" windowWidth="34660" windowHeight="19780" activeTab="3" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="32840" yWindow="4060" windowWidth="34660" windowHeight="19780" activeTab="3" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>

</xml_diff>